<commit_message>
update BOM and assembly process pictures
</commit_message>
<xml_diff>
--- a/BOM/MechanicalBOM.xlsx
+++ b/BOM/MechanicalBOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\模型\谐波赤道仪\GitHub\DIY-Harmonic-Equatorial-Mount\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\DIY-Harmonic-Equatorial-Mount\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D2B963D-A8AC-465D-86A0-7B30C24DDC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95545E11-89DC-4201-9BA2-AC5B55829123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="115">
   <si>
     <t>名称</t>
   </si>
@@ -39,12 +39,6 @@
     <t>塞打螺栓</t>
   </si>
   <si>
-    <t>8*10*M6</t>
-  </si>
-  <si>
-    <t>8*8*M6</t>
-  </si>
-  <si>
     <t>一字塞打螺栓</t>
   </si>
   <si>
@@ -54,74 +48,428 @@
     <t>M5*18</t>
   </si>
   <si>
+    <t>Φ12*25*M6</t>
+  </si>
+  <si>
+    <t>F8-14M 尺寸8*14*4</t>
+  </si>
+  <si>
+    <t>8-15(27*4/8*12*15)-圆光</t>
+  </si>
+  <si>
+    <t>M3*4</t>
+  </si>
+  <si>
+    <t>铜垫片</t>
+  </si>
+  <si>
+    <t>M8*12*0.5</t>
+  </si>
+  <si>
+    <t>M5*9*0.5</t>
+  </si>
+  <si>
+    <t>不锈钢超薄垫片</t>
+  </si>
+  <si>
+    <t>12.9级薄头内六角螺丝DIN7984</t>
+  </si>
+  <si>
+    <t>M4*16</t>
+  </si>
+  <si>
+    <t>M4*12</t>
+  </si>
+  <si>
+    <t>M6*12</t>
+  </si>
+  <si>
+    <t>纬度座部分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=706829568952&amp;mi_id=0000xv_Hkuuoo3E0Fx7SKdPJoKZA4qAK6yzxpGzK5hlaqis&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5886571346823</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=601075915248&amp;mi_id=0000surJTBGn5hJ-p1p08IDz8td8eT7gAx9Qm2uD4AG_Sag&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5681343815429</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=601075915248&amp;mi_id=0000surJTBGn5hJ-p1p08IDz8td8eT7gAx9Qm2uD4AG_Sag&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5790216147369</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=636950471592&amp;mi_id=0000jlLHgLAAC0JKaklJrW4BHuGyKZI3l-NZZQwgtDYO0PI&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=4572720393404</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>304不锈钢内螺纹圆柱销</t>
-  </si>
-  <si>
-    <t>Φ12*25*M6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=597217503705&amp;mi_id=0000BsPm9IddAblaEkLqg4m4C9OHKXGBuNi3uEpmxC3wtD0&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5510229308653</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>小微型推力球平面轴承</t>
-  </si>
-  <si>
-    <t>F8-14M 尺寸8*14*4</t>
-  </si>
-  <si>
-    <t>304不锈钢一字塞打螺丝</t>
-  </si>
-  <si>
-    <t>M8*4*M6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=586706057051&amp;mi_id=0000ciu5sZGunvTPl2eb_yXIN5aV9dSuRyU_GI8RATdzMuA&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5729732388208</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢一字开槽轴位螺丝钉</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>φ6*6(M5*6)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=632002464537&amp;mi_id=0000088g_i0X-nARhAksDKiA-OsufbvzwCcPlMrMVqe_pu0&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5559277728820</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>圆切边法兰铜合金无油衬套黄铜铜套</t>
-  </si>
-  <si>
-    <t>8-15(27*4/8*12*15)-圆光</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=561388884402&amp;mi_id=0000Q9Es8ZmOre8pNPLiDDDXphEUVindKIWt499U16dNy6o&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>M5*14</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=587639753812&amp;mi_id=0000cGhFpUF4WLFZ0-bbQ-uBY4v1NySu1sld_BE1MlPGugE&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=4942038499904</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>薄头内六角螺丝钉DIN7984</t>
-  </si>
-  <si>
-    <t>M3*4</t>
-  </si>
-  <si>
-    <t>铜垫片</t>
-  </si>
-  <si>
-    <t>M8*12*0.5</t>
-  </si>
-  <si>
-    <t>M5*9*0.5</t>
-  </si>
-  <si>
-    <t>不锈钢超薄垫片</t>
-  </si>
-  <si>
-    <t>8*12*0.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=611120761311&amp;mi_id=0000qD0BJTghbX-nCt7exgMTvZRQBfJTmPhNn-Ls2bdCsdk&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=4924269517558</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=626549373648&amp;mi_id=0000ffOAmkUrwxm4RWRnoDrV_Bky2tUHGeYV5WcP7QTJIPU&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=610746766031&amp;mi_id=0000Bb0eHT6T8fyS0T1_OeJioj7FsFHCu5uxVsjjpljuCJ4&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>12.9级薄头内六角螺丝DIN7984</t>
-  </si>
-  <si>
-    <t>M4*16</t>
-  </si>
-  <si>
-    <t>M4*12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=600935021724&amp;mi_id=0000j0HgLgN-0Jrp9lnXfmz0v8FqRVnK9a_pG0uv8McLHWE&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>12.9级高强度镀镍薄头内六角螺丝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=852888071845&amp;mi_id=0000GIlJj8suyPh8mlKGQ3kA6agK99o-I8WyklenHaMj2u4&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=625341852315&amp;mi_id=000076GZmldqNpTtASEDazl9WEpRskxQNjHalhHfMwoIFvQ&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>带钩拉簧</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0.8*5*20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢家具大平头倒边内六角螺丝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=859903073791&amp;mi_id=0000taNTRBsld1TVG21o8IxOLNlrsTAuX5uFX2doN8G1w-4&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>M6*12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢圆柱销销钉</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3*18</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=587625731480&amp;mi_id=0000wq9A60RwA5Ywsu7-pynUgHHm6aRX4-TBMMS9mb3wisY&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢薄头内六角螺丝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M6*14</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=15880165683&amp;mi_id=0000LXWRZTrC32hzl18vs9a30RhCG-KPrZmuMmasC11pacU&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>赤道仪部分</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢薄头内六角螺丝钉DIN7984</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3*10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=611120761311&amp;mi_id=0000qD0BJTghbX-nCt7exgMTvUwe1xQAcSiBA3lZ2HBlasY&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>塞打螺栓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M8*10*M6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M8*8*M6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M8*12*0.1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M8*12*0.2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>铝合金四方六面螺母</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>15*15*15-M5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=734244001867&amp;mi_id=0000oDysK6ARJnY0fI0ZOgwySjitxZsXg6Iea_EaIwelDNc&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=734244001867&amp;mi_id=0000oDysK6ARJnY0fI0ZOgwySjitxZsXg6Iea_EaIwelDNc&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5096386476347</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10*10*10-M4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M4*8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=743652912113&amp;mi_id=0000v9REBziiIcpxh9BHCC5eBxl66ri1uJVQ-7rE6JX0hgY&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M6*8</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢圆头内六角螺丝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=587776166655&amp;mi_id=00009IIyxmkO4s4oKlOYW6mKewptV8PvRl4djMyWhaMtENk&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>内六角螺丝12.9级高强度镀镍杯头螺栓</t>
+  </si>
+  <si>
+    <t>内六角螺丝12.9级高强度镀镍杯头螺栓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M4*45半牙</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=621643553473&amp;mi_id=00009U7wzAwL1s-2UVNdus86LI_N29MRv_D-QoW3A0C1yGo&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M4*40半牙</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304/316不锈钢尼龙锁紧螺母</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=556902193652&amp;mi_id=0000p1rVB25YXPayfR84Nm4ErTn6_sDAY4YQdrFOVyWpjvw&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=1013711773809&amp;mi_id=0000G-0vBAGPxmHHL3ueTXoF39FKaRH55khgxbwQtB8fV-M&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢螺母</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>六角铜柱单头铜螺柱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3*25+4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=601878143598&amp;mi_id=0000XOkgITD7jCt4FHKoGc3Ch7HFDXqSybh1TIg9__HiHDs&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=601878143598&amp;mi_id=0000XOkgITD7jCt4FHKoGc3Ch7HFDXqSybh1TIg9__HiHDs&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3*15+3</t>
+  </si>
+  <si>
+    <t>12.9级半牙内六角螺丝</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3*45</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=695021175011&amp;mi_id=0000-l2i3B2sDgpUth6n3cYbAMftyjrwW2bX4--ZrUuNk3Q&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=621643553473&amp;mi_id=00009U7wzAwL1s-2UVNdus86LMUskbjnesznFVVHJra7OEc&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M4*20</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>304不锈钢牙条细牙丝杆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M8*120</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=862294829769&amp;mi_id=0000ZaVMIpmG5PlKR1zoZA874wKt7aUwDOeA2ecbEWZPqc0&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c&amp;skuId=5680688716227</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>梅花手拧螺栓</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M6x45mm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=973695181639&amp;mi_id=0000OFU8l_mXziLXfT7t-Ucme5qL2loXEEW8CEHJfsufJmA&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RN方形四方防松锁紧螺母螺</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RN-M8*1.0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?ali_refid=a3_420434_1006%3A1150714776%3AH%3AewheRLpYki9xHqHTY%2FFj9w%3D%3D%3Addc27389fe7606c30299c8967ceb7956&amp;ali_trackid=282_ddc27389fe7606c30299c8967ceb7956&amp;id=783110990634&amp;mi_id=0000WGwij5I4xbGuvkjL_q1OEB7vTMz-gw0QBljgqDfQz80&amp;mm_sceneid=1_0_121666761_0&amp;priceTId=214782d617808419164568660e104b&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%22ef40f343d2aa9f9a393d53667fb1c3d3%22%7D&amp;xxc=ad_ztc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=833619009457&amp;mi_id=0000A1B8DT1VXEozYAtnUuIgFiZoHR5a4bj2klRcuu_HfiA&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>圆轴5×4.5mm</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>步进电机电磁制动器弹簧挤压机械刹车12v</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>雷赛电机42CM06</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?abbucket=11&amp;id=670665930208&amp;mi_id=0000PZjTCO_i8FY5r-kA57GsEFSiaAh2IMkB5MplRzbfqdE&amp;ns=1&amp;priceTId=214782d617808421678653457e104b&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%2224554e1d7e2553cdff12d4bdd37118b1%22%7D&amp;xxc=taobaoSearch</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>双轴电机42CM06-SZ/47高度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?abbucket=11&amp;id=670665930208&amp;mi_id=0000PZjTCO_i8FY5r-kA57GsEFSiaAh2IMkB5MplRzbfqdE&amp;ns=1&amp;priceTId=214782d617808421678653457e104b&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%2224554e1d7e2553cdff12d4bdd37118b1%22%7D&amp;xxc=taobaoSearch&amp;skuId=4999780927826</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>单轴电机42CM06-SZ/47高度</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>槽型形光电开关</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NPN</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=742487483554&amp;mi_id=0000M4geIl2ii2o-AkbDc9Rw04EejLbynMHg_LU6pa2-7uI&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,6 +482,14 @@
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="等线"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -154,17 +510,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -442,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
@@ -450,195 +815,695 @@
     <col min="3" max="3" width="11.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="C3" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>4</v>
+        <v>61</v>
       </c>
       <c r="C4" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1">
+        <v>8</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="1">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="C5" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="C9" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C10" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D10" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D13" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C14" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D14" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="C16" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="C17" s="1">
         <v>4</v>
       </c>
+      <c r="D17" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="1">
+        <v>8</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="1">
+        <v>4</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="1">
+        <v>4</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="1">
+        <v>4</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="1">
+        <v>4</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="1">
+        <v>4</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="1">
+        <v>2</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="1">
+        <v>2</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="1">
+        <v>8</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="1">
+        <v>2</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="1">
+        <v>4</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="1">
+        <v>16</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="1">
+        <v>16</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C35" s="1">
+        <v>10</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" s="1">
+        <v>4</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="1">
+        <v>24</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="1">
+        <v>24</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C39" s="1">
+        <v>6</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" s="1">
+        <v>4</v>
+      </c>
+      <c r="D40" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C41" s="1">
+        <v>4</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C42" s="1">
+        <v>25</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C43" s="1">
+        <v>6</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C44" s="1">
+        <v>1</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C45" s="1">
+        <v>1</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C46" s="1">
+        <v>1</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="1">
+        <v>4</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>114</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A28:C28"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{572BC529-0601-44E1-9C6E-8464481AF352}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{0A8938B4-BD8E-4C87-89EF-75C27E22CE81}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{B276E143-2468-4CBA-823B-245DCA4C69EC}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{BA9F555D-F20B-4BF8-9308-FFBB3EA9617E}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{14B27028-824F-4405-8938-BD16E8187CB0}"/>
+    <hyperlink ref="D9" r:id="rId6" xr:uid="{8F9E5CF6-C986-4109-A708-A23E64FDD104}"/>
+    <hyperlink ref="D10" r:id="rId7" xr:uid="{C59AEB1A-6B70-4E1B-A1AA-92FC50CE2581}"/>
+    <hyperlink ref="D11" r:id="rId8" xr:uid="{6D68D2CF-A5E5-4A64-9D38-1CF17D572552}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{8694EEDE-FF85-4D93-AEE2-18CFAD1A31B8}"/>
+    <hyperlink ref="D13" r:id="rId10" xr:uid="{F89D6FD0-F9AA-4601-99C0-DDF374D10621}"/>
+    <hyperlink ref="D15" r:id="rId11" xr:uid="{107A4C12-7EC8-492F-A152-CF36B75348C1}"/>
+    <hyperlink ref="D14" r:id="rId12" xr:uid="{3E19F28B-A4AC-4427-A5BD-F50550079906}"/>
+    <hyperlink ref="D16" r:id="rId13" xr:uid="{BA6B103E-F516-40FC-A003-9C09D804BDCF}"/>
+    <hyperlink ref="D17" r:id="rId14" xr:uid="{1EBC8E2C-8FDE-495C-BEE3-8E019F256CD3}"/>
+    <hyperlink ref="D18" r:id="rId15" xr:uid="{DDE12F3A-48C3-4C6F-866F-8F7188BCF204}"/>
+    <hyperlink ref="D19" r:id="rId16" xr:uid="{6BCA896C-A02A-421C-91CB-91F15B11ACEF}"/>
+    <hyperlink ref="D20" r:id="rId17" xr:uid="{8CFE9461-E3B8-47C9-B096-1A201536939D}"/>
+    <hyperlink ref="D21" r:id="rId18" xr:uid="{622F085A-2B48-43B1-871C-AEC509158010}"/>
+    <hyperlink ref="D7" r:id="rId19" xr:uid="{F6F39FCB-D4D5-4E97-AF4D-D56F64E092AD}"/>
+    <hyperlink ref="D22" r:id="rId20" xr:uid="{D7D1A1D6-B0CA-4942-A0CE-89FF2C4AA830}"/>
+    <hyperlink ref="D23" r:id="rId21" xr:uid="{1BD862E6-C481-484B-8791-7BEBCF1BC397}"/>
+    <hyperlink ref="D24" r:id="rId22" xr:uid="{B986D0C2-CC1C-48D5-B1FB-DF22750CED2F}"/>
+    <hyperlink ref="D30" r:id="rId23" xr:uid="{3AB49DB4-CEFB-4541-B70D-6D27AA44202F}"/>
+    <hyperlink ref="D31" r:id="rId24" xr:uid="{299F99AE-121A-41F9-9A1B-8AB5397E8E48}"/>
+    <hyperlink ref="D32" r:id="rId25" xr:uid="{0DCDD031-D08B-4E22-A551-34B2BC0D7C71}"/>
+    <hyperlink ref="D33" r:id="rId26" xr:uid="{0F922F0A-D46F-4CA2-A208-15881DCB4FEE}"/>
+    <hyperlink ref="D34" r:id="rId27" xr:uid="{96C69AC4-F6AC-4D1B-8125-FBFB3FD018F0}"/>
+    <hyperlink ref="D36" r:id="rId28" xr:uid="{2CF21C2E-B464-45B7-9811-2941DBD568CB}"/>
+    <hyperlink ref="D37" r:id="rId29" xr:uid="{3F3E30AC-AE2C-47D1-A831-3CD66D8A5195}"/>
+    <hyperlink ref="D38" r:id="rId30" xr:uid="{4640A412-940A-4761-BEB9-A671752E2F6F}"/>
+    <hyperlink ref="D35" r:id="rId31" xr:uid="{428E5E56-9EDE-4CDA-A035-613AE0276E72}"/>
+    <hyperlink ref="D39" r:id="rId32" xr:uid="{EC2BA01B-6F38-4A9E-A7E3-83FD138C5F1C}"/>
+    <hyperlink ref="D41" r:id="rId33" xr:uid="{9A55E747-B87F-4292-8C97-991505F7DE1D}"/>
+    <hyperlink ref="D42" r:id="rId34" xr:uid="{1354B794-7AA9-4268-950A-F5A87685129B}"/>
+    <hyperlink ref="D26" r:id="rId35" xr:uid="{59BD94A7-C326-4898-ACD0-AB06539C8B40}"/>
+    <hyperlink ref="D27" r:id="rId36" xr:uid="{B6C53113-0F09-4392-84BE-84CF7D075DCB}"/>
+    <hyperlink ref="D25" r:id="rId37" display="https://item.taobao.com/item.htm?ali_refid=a3_420434_1006%3A1150714776%3AH%3AewheRLpYki9xHqHTY%2FFj9w%3D%3D%3Addc27389fe7606c30299c8967ceb7956&amp;ali_trackid=282_ddc27389fe7606c30299c8967ceb7956&amp;id=783110990634&amp;mi_id=0000WGwij5I4xbGuvkjL_q1OEB7vTMz-gw0QBljgqDfQz80&amp;mm_sceneid=1_0_121666761_0&amp;priceTId=214782d617808419164568660e104b&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%22ef40f343d2aa9f9a393d53667fb1c3d3%22%7D&amp;xxc=ad_ztc" xr:uid="{7D7A5F6F-64B8-412A-A9C5-7C228F4B0DB7}"/>
+    <hyperlink ref="D43" r:id="rId38" xr:uid="{DBDDA5AD-67D4-4690-8216-79849787CF99}"/>
+    <hyperlink ref="D44" r:id="rId39" xr:uid="{5234CF3E-8FDE-402B-896B-F4BFCE44AD24}"/>
+    <hyperlink ref="D45" r:id="rId40" display="https://item.taobao.com/item.htm?abbucket=11&amp;id=670665930208&amp;mi_id=0000PZjTCO_i8FY5r-kA57GsEFSiaAh2IMkB5MplRzbfqdE&amp;ns=1&amp;priceTId=214782d617808421678653457e104b&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%2224554e1d7e2553cdff12d4bdd37118b1%22%7D&amp;xxc=taobaoSearch" xr:uid="{DD570655-1759-4C85-82E5-E02F5BE402B6}"/>
+    <hyperlink ref="D46" r:id="rId41" display="https://item.taobao.com/item.htm?abbucket=11&amp;id=670665930208&amp;mi_id=0000PZjTCO_i8FY5r-kA57GsEFSiaAh2IMkB5MplRzbfqdE&amp;ns=1&amp;priceTId=214782d617808421678653457e104b&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%2224554e1d7e2553cdff12d4bdd37118b1%22%7D&amp;xxc=taobaoSearch&amp;skuId=4999780927826" xr:uid="{B846C8F2-6E49-45AA-A36A-084CDB305853}"/>
+    <hyperlink ref="D47" r:id="rId42" xr:uid="{DEF290C6-F666-4709-A7A8-E3B5E683876A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update BOM and assembly guide
</commit_message>
<xml_diff>
--- a/BOM/MechanicalBOM.xlsx
+++ b/BOM/MechanicalBOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\DIY-Harmonic-Equatorial-Mount\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95545E11-89DC-4201-9BA2-AC5B55829123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{721770A5-45A3-43A7-8623-6D25C670FCC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="118">
   <si>
     <t>名称</t>
   </si>
@@ -462,6 +462,18 @@
   </si>
   <si>
     <t>https://detail.tmall.com/item.htm?id=742487483554&amp;mi_id=0000M4geIl2ii2o-AkbDc9Rw04EejLbynMHg_LU6pa2-7uI&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.77052e8dsXZo8c</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>土八热熔螺母</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>M3*6*4.6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?id=809364062256&amp;mi_id=0000As92SYpxzsWOMBX9WGOQwDxRzIEs8t2WRQKXTUry7Es&amp;spm=tbpc.boughtlist.suborder_itemtitle.1.18842e8d3wzrTj</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -519,12 +531,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -807,7 +819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
@@ -816,11 +828,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -843,7 +855,7 @@
       <c r="C3" s="1">
         <v>2</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -857,7 +869,7 @@
       <c r="C4" s="1">
         <v>2</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -871,7 +883,7 @@
       <c r="C5" s="1">
         <v>2</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -885,7 +897,7 @@
       <c r="C6" s="1">
         <v>8</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -899,7 +911,7 @@
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>47</v>
       </c>
     </row>
@@ -913,7 +925,7 @@
       <c r="C8" s="1">
         <v>1</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -927,7 +939,7 @@
       <c r="C9" s="1">
         <v>2</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
     </row>
@@ -941,7 +953,7 @@
       <c r="C10" s="1">
         <v>2</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>30</v>
       </c>
     </row>
@@ -955,7 +967,7 @@
       <c r="C11" s="1">
         <v>2</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -969,7 +981,7 @@
       <c r="C12" s="1">
         <v>2</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>34</v>
       </c>
     </row>
@@ -983,7 +995,7 @@
       <c r="C13" s="1">
         <v>4</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>36</v>
       </c>
     </row>
@@ -997,7 +1009,7 @@
       <c r="C14" s="1">
         <v>4</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1011,7 +1023,7 @@
       <c r="C15" s="1">
         <v>2</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1025,7 +1037,7 @@
       <c r="C16" s="1">
         <v>4</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="2" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1039,7 +1051,7 @@
       <c r="C17" s="1">
         <v>4</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="2" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1053,7 +1065,7 @@
       <c r="C18" s="1">
         <v>8</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1067,7 +1079,7 @@
       <c r="C19" s="1">
         <v>4</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1081,7 +1093,7 @@
       <c r="C20" s="1">
         <v>4</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1095,7 +1107,7 @@
       <c r="C21" s="1">
         <v>4</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1109,7 +1121,7 @@
       <c r="C22" s="1">
         <v>4</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D22" s="2" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1123,7 +1135,7 @@
       <c r="C23" s="1">
         <v>2</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="2" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1137,7 +1149,7 @@
       <c r="C24" s="1">
         <v>4</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="2" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1151,7 +1163,7 @@
       <c r="C25" s="1">
         <v>2</v>
       </c>
-      <c r="D25" s="3" t="s">
+      <c r="D25" s="2" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1165,7 +1177,7 @@
       <c r="C26" s="1">
         <v>1</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="2" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1179,17 +1191,17 @@
       <c r="C27" s="1">
         <v>2</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="2" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="3"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
@@ -1212,7 +1224,7 @@
       <c r="C30" s="1">
         <v>8</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1226,7 +1238,7 @@
       <c r="C31" s="1">
         <v>2</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1240,7 +1252,7 @@
       <c r="C32" s="1">
         <v>4</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="2" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1254,7 +1266,7 @@
       <c r="C33" s="1">
         <v>16</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="2" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1268,7 +1280,7 @@
       <c r="C34" s="1">
         <v>16</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="2" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1282,7 +1294,7 @@
       <c r="C35" s="1">
         <v>10</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="2" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1296,7 +1308,7 @@
       <c r="C36" s="1">
         <v>4</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="2" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1310,7 +1322,7 @@
       <c r="C37" s="1">
         <v>24</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="2" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1324,7 +1336,7 @@
       <c r="C38" s="1">
         <v>24</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="2" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1338,7 +1350,7 @@
       <c r="C39" s="1">
         <v>6</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="2" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1366,7 +1378,7 @@
       <c r="C41" s="1">
         <v>4</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="2" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1380,7 +1392,7 @@
       <c r="C42" s="1">
         <v>25</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1394,7 +1406,7 @@
       <c r="C43" s="1">
         <v>6</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1408,7 +1420,7 @@
       <c r="C44" s="1">
         <v>1</v>
       </c>
-      <c r="D44" s="3" t="s">
+      <c r="D44" s="2" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1416,13 +1428,13 @@
       <c r="A45" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C45" s="1">
         <v>1</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="D45" s="2" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1430,13 +1442,13 @@
       <c r="A46" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B46" s="3" t="s">
         <v>111</v>
       </c>
       <c r="C46" s="1">
         <v>1</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="D46" s="2" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1450,8 +1462,22 @@
       <c r="C47" s="1">
         <v>4</v>
       </c>
-      <c r="D47" s="3" t="s">
+      <c r="D47" s="2" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C48" s="1">
+        <v>10</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -1503,6 +1529,7 @@
     <hyperlink ref="D45" r:id="rId40" display="https://item.taobao.com/item.htm?abbucket=11&amp;id=670665930208&amp;mi_id=0000PZjTCO_i8FY5r-kA57GsEFSiaAh2IMkB5MplRzbfqdE&amp;ns=1&amp;priceTId=214782d617808421678653457e104b&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%2224554e1d7e2553cdff12d4bdd37118b1%22%7D&amp;xxc=taobaoSearch" xr:uid="{DD570655-1759-4C85-82E5-E02F5BE402B6}"/>
     <hyperlink ref="D46" r:id="rId41" display="https://item.taobao.com/item.htm?abbucket=11&amp;id=670665930208&amp;mi_id=0000PZjTCO_i8FY5r-kA57GsEFSiaAh2IMkB5MplRzbfqdE&amp;ns=1&amp;priceTId=214782d617808421678653457e104b&amp;spm=a21n57.1.hoverItem.11&amp;utparam=%7B%22aplus_abtest%22%3A%2224554e1d7e2553cdff12d4bdd37118b1%22%7D&amp;xxc=taobaoSearch&amp;skuId=4999780927826" xr:uid="{B846C8F2-6E49-45AA-A36A-084CDB305853}"/>
     <hyperlink ref="D47" r:id="rId42" xr:uid="{DEF290C6-F666-4709-A7A8-E3B5E683876A}"/>
+    <hyperlink ref="D48" r:id="rId43" xr:uid="{8F2D9626-A953-4E85-BD38-7429A3C79CEA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>